<commit_message>
update figure folder name, Q-Q plot labels
</commit_message>
<xml_diff>
--- a/data_080_human_digital_error_measure/digitized.xlsx
+++ b/data_080_human_digital_error_measure/digitized.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\gitgit\032 teMatDb1.1.6 to csv and filter  -- 20250514\data_80_human_digital_error_measure\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e64a25058d50c5c4/OneD-2025/8 pykeri proto code/032 teMatDb1.1.6 to csv and filter  -- 20250524/data_080_human_digital_error_measure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FDDC33-5A79-4CED-B8DA-7823CCBB5885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{E9FDDC33-5A79-4CED-B8DA-7823CCBB5885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{162935A2-24F3-4EC8-B138-2DD5569F7566}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{66D9F2D1-873E-42BC-A5D6-0895A02BEFDC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" activeTab="2" xr2:uid="{66D9F2D1-873E-42BC-A5D6-0895A02BEFDC}"/>
   </bookViews>
   <sheets>
     <sheet name="image used" sheetId="3" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="47">
   <si>
     <t>blue_square</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -242,6 +242,10 @@
   </si>
   <si>
     <t>2) reciprocal effects</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dpi low</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -728,9 +732,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -768,7 +772,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -874,7 +878,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1016,7 +1020,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1025,9 +1029,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{051D6DC6-1497-4CB7-9949-6EA3EB8E247F}">
   <dimension ref="D5:J5"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="5" spans="4:10" x14ac:dyDescent="0.6">
+    <row r="5" spans="4:10" x14ac:dyDescent="0.45">
       <c r="D5" t="s">
         <v>17</v>
       </c>
@@ -1045,14 +1049,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A61D2C-BF7B-4983-AA9E-6B55C107996D}">
   <dimension ref="B4:AL36"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="15" width="5.75" customWidth="1"/>
     <col min="17" max="25" width="5.75" customWidth="1"/>
     <col min="28" max="35" width="5.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="4" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -1121,7 +1125,7 @@
       <c r="AH4" s="1"/>
       <c r="AI4" s="1"/>
     </row>
-    <row r="5" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:38" x14ac:dyDescent="0.45">
       <c r="G5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1181,7 +1185,7 @@
       <c r="AH5" s="1"/>
       <c r="AI5" s="1"/>
     </row>
-    <row r="6" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="6" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1270,7 +1274,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="7" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B7" s="1">
         <v>0.61929109000000004</v>
       </c>
@@ -1367,7 +1371,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="8" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B8" s="1">
         <v>1.01005926</v>
       </c>
@@ -1483,7 +1487,7 @@
         <v>-0.18311212104443675</v>
       </c>
     </row>
-    <row r="9" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="9" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
         <v>5.9755596600000001</v>
       </c>
@@ -1599,7 +1603,7 @@
         <v>0.26657333513867226</v>
       </c>
     </row>
-    <row r="10" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="10" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B10" s="1">
         <v>7.5932600099999998</v>
       </c>
@@ -1680,7 +1684,7 @@
       <c r="AH10" s="1"/>
       <c r="AI10" s="1"/>
     </row>
-    <row r="11" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="11" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B11" s="1">
         <v>7.8804391100000002</v>
       </c>
@@ -1786,7 +1790,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="12" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B12" s="1">
         <v>18.96126589</v>
       </c>
@@ -1902,7 +1906,7 @@
         <v>-1.8311212104443675E-3</v>
       </c>
     </row>
-    <row r="13" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="13" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B13" s="1">
         <v>27.488892379999999</v>
       </c>
@@ -2018,7 +2022,7 @@
         <v>2.6657333513867227E-3</v>
       </c>
     </row>
-    <row r="14" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="14" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B14" s="1">
         <v>33.628172839999998</v>
       </c>
@@ -2097,7 +2101,7 @@
       <c r="AH14" s="1"/>
       <c r="AI14" s="1"/>
     </row>
-    <row r="15" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="15" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B15" s="1">
         <v>34.344647449999997</v>
       </c>
@@ -2185,7 +2189,7 @@
       </c>
       <c r="AI15" s="1"/>
     </row>
-    <row r="16" spans="2:38" x14ac:dyDescent="0.6">
+    <row r="16" spans="2:38" x14ac:dyDescent="0.45">
       <c r="B16" s="1">
         <v>34.655171420000002</v>
       </c>
@@ -2273,7 +2277,7 @@
       </c>
       <c r="AI16" s="1"/>
     </row>
-    <row r="17" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="17" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B17" s="1">
         <v>35.427304530000001</v>
       </c>
@@ -2368,7 +2372,7 @@
         <v>-3.9324960886337891E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="18" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B18" s="1">
         <v>39.17994487</v>
       </c>
@@ -2463,7 +2467,7 @@
         <v>0.2311359068316696</v>
       </c>
     </row>
-    <row r="19" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="19" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B19" s="1">
         <v>45.118863169999997</v>
       </c>
@@ -2544,7 +2548,7 @@
       <c r="AH19" s="1"/>
       <c r="AI19" s="1"/>
     </row>
-    <row r="20" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="20" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B20" s="1">
         <v>45.90439207</v>
       </c>
@@ -2625,7 +2629,7 @@
       <c r="AH20" s="1"/>
       <c r="AI20" s="1"/>
     </row>
-    <row r="21" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="21" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B21" s="1">
         <v>50.232937120000003</v>
       </c>
@@ -2706,7 +2710,7 @@
       <c r="AH21" s="1"/>
       <c r="AI21" s="1"/>
     </row>
-    <row r="22" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="22" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B22" s="1">
         <v>52.973726739999996</v>
       </c>
@@ -2787,7 +2791,7 @@
       <c r="AH22" s="1"/>
       <c r="AI22" s="1"/>
     </row>
-    <row r="23" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="23" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B23" s="1">
         <v>58.012670819999997</v>
       </c>
@@ -2868,7 +2872,7 @@
       <c r="AH23" s="1"/>
       <c r="AI23" s="1"/>
     </row>
-    <row r="24" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="24" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B24" s="1">
         <v>62.685176329999997</v>
       </c>
@@ -2949,7 +2953,7 @@
       <c r="AH24" s="1"/>
       <c r="AI24" s="1"/>
     </row>
-    <row r="25" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="25" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B25" s="1">
         <v>63.242376</v>
       </c>
@@ -3030,7 +3034,7 @@
       <c r="AH25" s="1"/>
       <c r="AI25" s="1"/>
     </row>
-    <row r="26" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="26" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B26" s="1">
         <v>68.567099420000005</v>
       </c>
@@ -3111,7 +3115,7 @@
       <c r="AH26" s="1"/>
       <c r="AI26" s="1"/>
     </row>
-    <row r="27" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="27" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B27" s="1">
         <v>70.527367060000003</v>
       </c>
@@ -3192,7 +3196,7 @@
       <c r="AH27" s="1"/>
       <c r="AI27" s="1"/>
     </row>
-    <row r="28" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="28" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B28" s="1">
         <v>73.09919721</v>
       </c>
@@ -3273,7 +3277,7 @@
       <c r="AH28" s="1"/>
       <c r="AI28" s="1"/>
     </row>
-    <row r="29" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="29" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B29" s="1">
         <v>74.649008069999994</v>
       </c>
@@ -3354,7 +3358,7 @@
       <c r="AH29" s="1"/>
       <c r="AI29" s="1"/>
     </row>
-    <row r="30" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="30" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B30" s="1">
         <v>75.305004940000003</v>
       </c>
@@ -3435,7 +3439,7 @@
       <c r="AH30" s="1"/>
       <c r="AI30" s="1"/>
     </row>
-    <row r="31" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="31" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B31" s="1">
         <v>83.516144100000005</v>
       </c>
@@ -3516,7 +3520,7 @@
       <c r="AH31" s="1"/>
       <c r="AI31" s="1"/>
     </row>
-    <row r="32" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="32" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B32" s="1">
         <v>84.433256999999998</v>
       </c>
@@ -3597,7 +3601,7 @@
       <c r="AH32" s="1"/>
       <c r="AI32" s="1"/>
     </row>
-    <row r="33" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="33" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B33" s="1">
         <v>92.083094310000007</v>
       </c>
@@ -3678,7 +3682,7 @@
       <c r="AH33" s="1"/>
       <c r="AI33" s="1"/>
     </row>
-    <row r="34" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="34" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B34" s="1">
         <v>94.165881420000005</v>
       </c>
@@ -3759,7 +3763,7 @@
       <c r="AH34" s="1"/>
       <c r="AI34" s="1"/>
     </row>
-    <row r="35" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="35" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B35" s="1">
         <v>97.159661510000007</v>
       </c>
@@ -3840,7 +3844,7 @@
       <c r="AH35" s="1"/>
       <c r="AI35" s="1"/>
     </row>
-    <row r="36" spans="2:35" x14ac:dyDescent="0.6">
+    <row r="36" spans="2:35" x14ac:dyDescent="0.45">
       <c r="B36" s="1">
         <v>99.480866559999996</v>
       </c>
@@ -3937,19 +3941,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AS39"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="23" width="5.75" customWidth="1"/>
     <col min="25" max="33" width="5.75" customWidth="1"/>
-    <col min="35" max="35" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="36" max="39" width="6.625" customWidth="1"/>
+    <col min="35" max="35" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="39" width="6.58203125" customWidth="1"/>
     <col min="40" max="40" width="6.5" customWidth="1"/>
-    <col min="41" max="41" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="42" max="45" width="6.625" customWidth="1"/>
-    <col min="46" max="46" width="4.3125" customWidth="1"/>
+    <col min="41" max="41" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="45" width="6.58203125" customWidth="1"/>
+    <col min="46" max="46" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -4051,7 +4055,7 @@
         <v>0.41036389330426926</v>
       </c>
     </row>
-    <row r="2" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -4153,7 +4157,7 @@
         <v>0.89299207951970061</v>
       </c>
     </row>
-    <row r="3" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -4254,7 +4258,7 @@
         <v>-9.1590545021801972E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -4355,7 +4359,7 @@
         <v>0.89299207951970061</v>
       </c>
     </row>
-    <row r="6" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:45" x14ac:dyDescent="0.45">
       <c r="Y6" t="s">
         <v>43</v>
       </c>
@@ -4376,7 +4380,7 @@
       <c r="AR6" s="6"/>
       <c r="AS6" s="6"/>
     </row>
-    <row r="7" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>0</v>
       </c>
@@ -4451,7 +4455,7 @@
       <c r="AR7" s="7"/>
       <c r="AS7" s="6"/>
     </row>
-    <row r="8" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:45" x14ac:dyDescent="0.45">
       <c r="N8" s="1" t="s">
         <v>14</v>
       </c>
@@ -4504,7 +4508,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
         <v>1</v>
       </c>
@@ -4600,19 +4604,19 @@
       <c r="AN9" s="1"/>
       <c r="AO9" s="8"/>
       <c r="AP9" s="9" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="AQ9" s="9" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="AR9" s="9" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="AS9" s="9" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B10" s="1">
         <v>0.61929109000000004</v>
       </c>
@@ -4728,7 +4732,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B11" s="1">
         <v>1.01005926</v>
       </c>
@@ -4856,7 +4860,7 @@
         <v>0.41036389330426926</v>
       </c>
     </row>
-    <row r="12" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B12" s="1">
         <v>5.9755596600000001</v>
       </c>
@@ -4983,7 +4987,7 @@
         <v>0.89299207951970061</v>
       </c>
     </row>
-    <row r="13" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B13" s="1">
         <v>7.5932600099999998</v>
       </c>
@@ -5111,7 +5115,7 @@
         <v>0.26219446936639113</v>
       </c>
     </row>
-    <row r="14" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B14" s="1">
         <v>7.8804391100000002</v>
       </c>
@@ -5200,7 +5204,7 @@
         <v>0.41437059323149938</v>
       </c>
     </row>
-    <row r="15" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B15" s="1">
         <v>18.96126589</v>
       </c>
@@ -5304,7 +5308,7 @@
       <c r="AR15" s="9"/>
       <c r="AS15" s="9"/>
     </row>
-    <row r="16" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B16" s="1">
         <v>27.488892379999999</v>
       </c>
@@ -5432,7 +5436,7 @@
         <v>98.253275109170303</v>
       </c>
     </row>
-    <row r="17" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="17" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B17" s="1">
         <v>33.628172839999998</v>
       </c>
@@ -5524,19 +5528,19 @@
         <v>38</v>
       </c>
       <c r="AJ17" s="12">
-        <f>AJ11/AJ$16</f>
+        <f t="shared" ref="AJ17:AM19" si="11">AJ11/AJ$16</f>
         <v>6.2193249727176723E-4</v>
       </c>
       <c r="AK17" s="12">
-        <f>AK11/AK$16</f>
+        <f t="shared" si="11"/>
         <v>5.2924374661365706E-4</v>
       </c>
       <c r="AL17" s="12">
-        <f>AL11/AL$16</f>
+        <f t="shared" si="11"/>
         <v>3.8785267279575455E-4</v>
       </c>
       <c r="AM17" s="12">
-        <f>AM11/AM$16</f>
+        <f t="shared" si="11"/>
         <v>3.0813553530232344E-3</v>
       </c>
       <c r="AN17" s="2"/>
@@ -5544,23 +5548,23 @@
         <v>38</v>
       </c>
       <c r="AP17" s="12">
-        <f>AP11/AP$16</f>
+        <f t="shared" ref="AP17:AS19" si="12">AP11/AP$16</f>
         <v>8.5398788929175369E-4</v>
       </c>
       <c r="AQ17" s="12">
-        <f>AQ11/AQ$16</f>
+        <f t="shared" si="12"/>
         <v>-3.361826503296323E-4</v>
       </c>
       <c r="AR17" s="12">
-        <f>AR11/AR$16</f>
+        <f t="shared" si="12"/>
         <v>6.5940146541006606E-4</v>
       </c>
       <c r="AS17" s="12">
-        <f>AS11/AS$16</f>
+        <f t="shared" si="12"/>
         <v>4.1765925140745631E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="18" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B18" s="1">
         <v>34.344647449999997</v>
       </c>
@@ -5652,19 +5656,19 @@
         <v>36</v>
       </c>
       <c r="AJ18" s="12">
-        <f>AJ12/AJ$16</f>
+        <f t="shared" si="11"/>
         <v>1.452731495843273E-3</v>
       </c>
       <c r="AK18" s="12">
-        <f>AK12/AK$16</f>
+        <f t="shared" si="11"/>
         <v>1.6130940765402622E-3</v>
       </c>
       <c r="AL18" s="12">
-        <f>AL12/AL$16</f>
+        <f t="shared" si="11"/>
         <v>1.583531408465864E-3</v>
       </c>
       <c r="AM18" s="12">
-        <f>AM12/AM$16</f>
+        <f t="shared" si="11"/>
         <v>4.1735706014145828E-3</v>
       </c>
       <c r="AN18" s="1"/>
@@ -5672,23 +5676,23 @@
         <v>36</v>
       </c>
       <c r="AP18" s="12">
-        <f>AP12/AP$16</f>
+        <f t="shared" si="12"/>
         <v>4.2587466621649269E-3</v>
       </c>
       <c r="AQ18" s="12">
-        <f>AQ12/AQ$16</f>
+        <f t="shared" si="12"/>
         <v>5.4011844302429323E-3</v>
       </c>
       <c r="AR18" s="12">
-        <f>AR12/AR$16</f>
+        <f t="shared" si="12"/>
         <v>2.9512778617513122E-3</v>
       </c>
       <c r="AS18" s="12">
-        <f>AS12/AS$16</f>
+        <f t="shared" si="12"/>
         <v>9.0886749426671749E-3</v>
       </c>
     </row>
-    <row r="19" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="19" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B19" s="1">
         <v>34.655171420000002</v>
       </c>
@@ -5780,19 +5784,19 @@
         <v>35</v>
       </c>
       <c r="AJ19" s="12">
-        <f>AJ13/AJ$16</f>
+        <f t="shared" si="11"/>
         <v>5.0189537839337992E-4</v>
       </c>
       <c r="AK19" s="12">
-        <f>AK13/AK$16</f>
+        <f t="shared" si="11"/>
         <v>5.3518083635148829E-4</v>
       </c>
       <c r="AL19" s="12">
-        <f>AL13/AL$16</f>
+        <f t="shared" si="11"/>
         <v>5.064618664839737E-4</v>
       </c>
       <c r="AM19" s="12">
-        <f>AM13/AM$16</f>
+        <f t="shared" si="11"/>
         <v>5.6706341312331033E-4</v>
       </c>
       <c r="AN19" s="2"/>
@@ -5800,23 +5804,23 @@
         <v>35</v>
       </c>
       <c r="AP19" s="12">
-        <f>AP13/AP$16</f>
+        <f t="shared" si="12"/>
         <v>2.0596620802885556E-3</v>
       </c>
       <c r="AQ19" s="12">
-        <f>AQ13/AQ$16</f>
+        <f t="shared" si="12"/>
         <v>2.9612168813543875E-3</v>
       </c>
       <c r="AR19" s="12">
-        <f>AR13/AR$16</f>
+        <f t="shared" si="12"/>
         <v>1.774058859269047E-3</v>
       </c>
       <c r="AS19" s="12">
-        <f>AS13/AS$16</f>
+        <f t="shared" si="12"/>
         <v>2.668557043773492E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="20" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B20" s="1">
         <v>35.427304530000001</v>
       </c>
@@ -5905,7 +5909,7 @@
         <v>0.60924741572053076</v>
       </c>
     </row>
-    <row r="21" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="21" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B21" s="1">
         <v>39.17994487</v>
       </c>
@@ -6033,7 +6037,7 @@
         <v>50.692867540029063</v>
       </c>
     </row>
-    <row r="22" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="22" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B22" s="1">
         <v>45.118863169999997</v>
       </c>
@@ -6125,19 +6129,19 @@
         <v>38</v>
       </c>
       <c r="AJ22" s="12">
-        <f>AJ11/AJ$21</f>
+        <f t="shared" ref="AJ22:AM24" si="13">AJ11/AJ$21</f>
         <v>1.2077339803639494E-3</v>
       </c>
       <c r="AK22" s="12">
-        <f>AK11/AK$21</f>
+        <f t="shared" si="13"/>
         <v>1.0638140445615467E-3</v>
       </c>
       <c r="AL22" s="12">
-        <f>AL11/AL$21</f>
+        <f t="shared" si="13"/>
         <v>7.7326462511052895E-4</v>
       </c>
       <c r="AM22" s="12">
-        <f>AM11/AM$21</f>
+        <f t="shared" si="13"/>
         <v>5.9712851477868615E-3</v>
       </c>
       <c r="AN22" s="2"/>
@@ -6145,23 +6149,23 @@
         <v>38</v>
       </c>
       <c r="AP22" s="12">
-        <f>AP11/AP$21</f>
+        <f t="shared" ref="AP22:AS24" si="14">AP11/AP$21</f>
         <v>1.6609805250479973E-3</v>
       </c>
       <c r="AQ22" s="12">
-        <f>AQ11/AQ$21</f>
+        <f t="shared" si="14"/>
         <v>-6.7442926059267194E-4</v>
       </c>
       <c r="AR22" s="12">
-        <f>AR11/AR$21</f>
+        <f t="shared" si="14"/>
         <v>1.3167802269385066E-3</v>
       </c>
       <c r="AS22" s="12">
-        <f>AS11/AS$21</f>
+        <f t="shared" si="14"/>
         <v>8.0951012088678938E-3</v>
       </c>
     </row>
-    <row r="23" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="23" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B23" s="1">
         <v>45.90439207</v>
       </c>
@@ -6253,19 +6257,19 @@
         <v>36</v>
       </c>
       <c r="AJ23" s="12">
-        <f>AJ12/AJ$21</f>
+        <f t="shared" si="13"/>
         <v>2.8210669157366719E-3</v>
       </c>
       <c r="AK23" s="12">
-        <f>AK12/AK$21</f>
+        <f t="shared" si="13"/>
         <v>3.2424230702819373E-3</v>
       </c>
       <c r="AL23" s="12">
-        <f>AL12/AL$21</f>
+        <f t="shared" si="13"/>
         <v>3.1570978023475606E-3</v>
       </c>
       <c r="AM23" s="12">
-        <f>AM12/AM$21</f>
+        <f t="shared" si="13"/>
         <v>8.0878630635753436E-3</v>
       </c>
       <c r="AN23" s="1"/>
@@ -6273,23 +6277,23 @@
         <v>36</v>
       </c>
       <c r="AP23" s="12">
-        <f>AP12/AP$21</f>
+        <f t="shared" si="14"/>
         <v>8.2831329995037804E-3</v>
       </c>
       <c r="AQ23" s="12">
-        <f>AQ12/AQ$21</f>
+        <f t="shared" si="14"/>
         <v>1.0835528894907732E-2</v>
       </c>
       <c r="AR23" s="12">
-        <f>AR12/AR$21</f>
+        <f t="shared" si="14"/>
         <v>5.8935027239267034E-3</v>
       </c>
       <c r="AS23" s="12">
-        <f>AS12/AS$21</f>
+        <f t="shared" si="14"/>
         <v>1.7615734182221184E-2</v>
       </c>
     </row>
-    <row r="24" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="24" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B24" s="1">
         <v>50.232937120000003</v>
       </c>
@@ -6381,19 +6385,19 @@
         <v>35</v>
       </c>
       <c r="AJ24" s="12">
-        <f>AJ13/AJ$21</f>
+        <f t="shared" si="13"/>
         <v>9.7463326925724869E-4</v>
       </c>
       <c r="AK24" s="12">
-        <f>AK13/AK$21</f>
+        <f t="shared" si="13"/>
         <v>1.075747977626112E-3</v>
       </c>
       <c r="AL24" s="12">
-        <f>AL13/AL$21</f>
+        <f t="shared" si="13"/>
         <v>1.009736615959181E-3</v>
       </c>
       <c r="AM24" s="12">
-        <f>AM13/AM$21</f>
+        <f t="shared" si="13"/>
         <v>1.0988986821381442E-3</v>
       </c>
       <c r="AN24" s="2"/>
@@ -6401,23 +6405,23 @@
         <v>35</v>
       </c>
       <c r="AP24" s="12">
-        <f>AP13/AP$21</f>
+        <f t="shared" si="14"/>
         <v>4.0059802327833431E-3</v>
       </c>
       <c r="AQ24" s="12">
-        <f>AQ13/AQ$21</f>
+        <f t="shared" si="14"/>
         <v>5.9406138591273508E-3</v>
       </c>
       <c r="AR24" s="12">
-        <f>AR13/AR$21</f>
+        <f t="shared" si="14"/>
         <v>3.5426758201967798E-3</v>
       </c>
       <c r="AS24" s="12">
-        <f>AS13/AS$21</f>
+        <f t="shared" si="14"/>
         <v>5.1722161733966255E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="25" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B25" s="1">
         <v>52.973726739999996</v>
       </c>
@@ -6506,7 +6510,7 @@
         <v>0.70991278524019208</v>
       </c>
     </row>
-    <row r="26" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="26" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B26" s="1">
         <v>58.012670819999997</v>
       </c>
@@ -6595,7 +6599,7 @@
         <v>0.89299207951970061</v>
       </c>
     </row>
-    <row r="27" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="27" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B27" s="1">
         <v>62.685176329999997</v>
       </c>
@@ -6684,7 +6688,7 @@
         <v>0.17329067934497999</v>
       </c>
     </row>
-    <row r="28" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="28" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B28" s="1">
         <v>63.242376</v>
       </c>
@@ -6781,7 +6785,7 @@
       <c r="AQ28" s="1"/>
       <c r="AR28" s="1"/>
     </row>
-    <row r="29" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="29" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B29" s="1">
         <v>68.567099420000005</v>
       </c>
@@ -6878,7 +6882,7 @@
       <c r="AQ29" s="1"/>
       <c r="AR29" s="1"/>
     </row>
-    <row r="30" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="30" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B30" s="1">
         <v>70.527367060000003</v>
       </c>
@@ -6975,7 +6979,7 @@
       <c r="AQ30" s="1"/>
       <c r="AR30" s="1"/>
     </row>
-    <row r="31" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="31" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B31" s="1">
         <v>73.09919721</v>
       </c>
@@ -7072,7 +7076,7 @@
       <c r="AQ31" s="1"/>
       <c r="AR31" s="1"/>
     </row>
-    <row r="32" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="32" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B32" s="1">
         <v>74.649008069999994</v>
       </c>
@@ -7169,7 +7173,7 @@
       <c r="AQ32" s="1"/>
       <c r="AR32" s="1"/>
     </row>
-    <row r="33" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="33" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B33" s="1">
         <v>75.305004940000003</v>
       </c>
@@ -7266,7 +7270,7 @@
       <c r="AQ33" s="1"/>
       <c r="AR33" s="1"/>
     </row>
-    <row r="34" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="34" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B34" s="1">
         <v>83.516144100000005</v>
       </c>
@@ -7363,7 +7367,7 @@
       <c r="AQ34" s="1"/>
       <c r="AR34" s="1"/>
     </row>
-    <row r="35" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="35" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B35" s="1">
         <v>84.433256999999998</v>
       </c>
@@ -7460,7 +7464,7 @@
       <c r="AQ35" s="1"/>
       <c r="AR35" s="1"/>
     </row>
-    <row r="36" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="36" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B36" s="1">
         <v>92.083094310000007</v>
       </c>
@@ -7557,7 +7561,7 @@
       <c r="AQ36" s="1"/>
       <c r="AR36" s="1"/>
     </row>
-    <row r="37" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="37" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B37" s="1">
         <v>94.165881420000005</v>
       </c>
@@ -7654,7 +7658,7 @@
       <c r="AQ37" s="1"/>
       <c r="AR37" s="1"/>
     </row>
-    <row r="38" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="38" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B38" s="1">
         <v>97.159661510000007</v>
       </c>
@@ -7751,7 +7755,7 @@
       <c r="AQ38" s="1"/>
       <c r="AR38" s="1"/>
     </row>
-    <row r="39" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="39" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B39" s="1">
         <v>99.480866559999996</v>
       </c>
@@ -7863,19 +7867,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AS39"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="23" width="5.75" customWidth="1"/>
     <col min="25" max="33" width="5.75" customWidth="1"/>
-    <col min="35" max="35" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="36" max="39" width="6.625" customWidth="1"/>
+    <col min="35" max="35" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="39" width="6.58203125" customWidth="1"/>
     <col min="40" max="40" width="6.5" customWidth="1"/>
-    <col min="41" max="41" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="42" max="45" width="6.625" customWidth="1"/>
-    <col min="46" max="46" width="4.3125" customWidth="1"/>
+    <col min="41" max="41" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="45" width="6.58203125" customWidth="1"/>
+    <col min="46" max="46" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -7976,7 +7980,7 @@
         <v>-9.2534973778789748E-2</v>
       </c>
     </row>
-    <row r="2" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -8077,7 +8081,7 @@
         <v>-2.5918663740169823E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -8178,7 +8182,7 @@
         <v>-0.87123591956983759</v>
       </c>
     </row>
-    <row r="4" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:45" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -8279,10 +8283,10 @@
         <v>0.87123591956983759</v>
       </c>
     </row>
-    <row r="5" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.45">
       <c r="AJ5" s="1"/>
     </row>
-    <row r="6" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:45" x14ac:dyDescent="0.45">
       <c r="Y6" t="s">
         <v>43</v>
       </c>
@@ -8303,7 +8307,7 @@
       <c r="AR6" s="6"/>
       <c r="AS6" s="6"/>
     </row>
-    <row r="7" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>0</v>
       </c>
@@ -8378,7 +8382,7 @@
       <c r="AR7" s="7"/>
       <c r="AS7" s="6"/>
     </row>
-    <row r="8" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:45" x14ac:dyDescent="0.45">
       <c r="N8" s="1" t="s">
         <v>14</v>
       </c>
@@ -8431,7 +8435,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
         <v>1</v>
       </c>
@@ -8539,7 +8543,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B10" s="1">
         <v>0.61929109000000004</v>
       </c>
@@ -8663,7 +8667,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B11" s="1">
         <v>1.01005926</v>
       </c>
@@ -8711,15 +8715,15 @@
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
       <c r="T11" s="1">
-        <f>100/N11</f>
+        <f t="shared" ref="T11:T25" si="17">100/N11</f>
         <v>107.92307692307725</v>
       </c>
       <c r="U11" s="1">
-        <f>100/O11</f>
+        <f t="shared" ref="U11:U25" si="18">100/O11</f>
         <v>2.4616935483870983</v>
       </c>
       <c r="V11" s="1">
-        <f t="shared" ref="V11:V39" si="17">100/P11</f>
+        <f t="shared" ref="V11:V39" si="19">100/P11</f>
         <v>9.9503546099291409</v>
       </c>
       <c r="W11" s="1">
@@ -8727,7 +8731,7 @@
         <v>6.0445544554455601</v>
       </c>
       <c r="Y11" s="1">
-        <f t="shared" ref="Y11:Y39" si="18">B11-N11</f>
+        <f t="shared" ref="Y11:Y39" si="20">B11-N11</f>
         <v>8.3473372615825991E-2</v>
       </c>
       <c r="Z11" s="1">
@@ -8744,7 +8748,7 @@
       </c>
       <c r="AC11" s="1"/>
       <c r="AD11" s="1">
-        <f t="shared" ref="AD11:AD39" si="19">H11-T11</f>
+        <f t="shared" ref="AD11:AD39" si="21">H11-T11</f>
         <v>-8.9189848265402532</v>
       </c>
       <c r="AE11" s="1">
@@ -8799,7 +8803,7 @@
         <v>-9.2534973778789748E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B12" s="1">
         <v>5.9755596600000001</v>
       </c>
@@ -8847,15 +8851,15 @@
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1">
-        <f>100/N12</f>
+        <f t="shared" si="17"/>
         <v>17.109756097561014</v>
       </c>
       <c r="U12" s="1">
-        <f>100/O12</f>
+        <f t="shared" si="18"/>
         <v>1.3954285714285728</v>
       </c>
       <c r="V12" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>7.794444444444502</v>
       </c>
       <c r="W12" s="1">
@@ -8863,7 +8867,7 @@
         <v>1.0158069883527459</v>
       </c>
       <c r="Y12" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.13094098573059032</v>
       </c>
       <c r="Z12" s="1">
@@ -8880,7 +8884,7 @@
       </c>
       <c r="AC12" s="1"/>
       <c r="AD12" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-0.37492192472305064</v>
       </c>
       <c r="AE12" s="1">
@@ -8934,7 +8938,7 @@
         <v>0.87123591956983759</v>
       </c>
     </row>
-    <row r="13" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B13" s="1">
         <v>7.5932600099999998</v>
       </c>
@@ -8982,15 +8986,15 @@
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1">
-        <f>100/N13</f>
+        <f t="shared" si="17"/>
         <v>13.361904761904771</v>
       </c>
       <c r="U13" s="1">
-        <f>100/O13</f>
+        <f t="shared" si="18"/>
         <v>1.8305847076461779</v>
       </c>
       <c r="V13" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>6.3198198198198581</v>
       </c>
       <c r="W13" s="1">
@@ -8998,7 +9002,7 @@
         <v>1.5167701863354044</v>
       </c>
       <c r="Y13" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.1092970734355001</v>
       </c>
       <c r="Z13" s="1">
@@ -9015,7 +9019,7 @@
       </c>
       <c r="AC13" s="1"/>
       <c r="AD13" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-0.19233070961309906</v>
       </c>
       <c r="AE13" s="1">
@@ -9070,7 +9074,7 @@
         <v>0.21241124810530118</v>
       </c>
     </row>
-    <row r="14" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B14" s="1">
         <v>7.8804391100000002</v>
       </c>
@@ -9118,15 +9122,15 @@
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1">
-        <f>100/N14</f>
+        <f t="shared" si="17"/>
         <v>12.75454545454545</v>
       </c>
       <c r="U14" s="1">
-        <f>100/O14</f>
+        <f t="shared" si="18"/>
         <v>26.543478260869758</v>
       </c>
       <c r="V14" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>5.8949579831932919</v>
       </c>
       <c r="W14" s="1">
@@ -9134,7 +9138,7 @@
         <v>8.912408759124105</v>
       </c>
       <c r="Y14" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>4.0096985980039968E-2</v>
       </c>
       <c r="Z14" s="1">
@@ -9151,7 +9155,7 @@
       </c>
       <c r="AC14" s="1"/>
       <c r="AD14" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-6.4897250411302565E-2</v>
       </c>
       <c r="AE14" s="1">
@@ -9167,7 +9171,7 @@
         <v>-0.22134671294990937</v>
       </c>
     </row>
-    <row r="15" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B15" s="1">
         <v>18.96126589</v>
       </c>
@@ -9215,15 +9219,15 @@
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1">
-        <f>100/N15</f>
+        <f t="shared" si="17"/>
         <v>5.314393939393967</v>
       </c>
       <c r="U15" s="1">
-        <f>100/O15</f>
+        <f t="shared" si="18"/>
         <v>1.0303797468354436</v>
       </c>
       <c r="V15" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>5.7975206611570274</v>
       </c>
       <c r="W15" s="1">
@@ -9231,7 +9235,7 @@
         <v>3.6017699115044333</v>
       </c>
       <c r="Y15" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.14444479235219987</v>
       </c>
       <c r="Z15" s="1">
@@ -9248,7 +9252,7 @@
       </c>
       <c r="AC15" s="1"/>
       <c r="AD15" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-4.0484455706008227E-2</v>
       </c>
       <c r="AE15" s="1">
@@ -9279,7 +9283,7 @@
       <c r="AR15" s="9"/>
       <c r="AS15" s="9"/>
     </row>
-    <row r="16" spans="1:45" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:45" x14ac:dyDescent="0.45">
       <c r="B16" s="1">
         <v>27.488892379999999</v>
       </c>
@@ -9327,15 +9331,15 @@
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1">
-        <f>100/N16</f>
+        <f t="shared" si="17"/>
         <v>3.6536458333333415</v>
       </c>
       <c r="U16" s="1">
-        <f>100/O16</f>
+        <f t="shared" si="18"/>
         <v>1.3657718120805371</v>
       </c>
       <c r="V16" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>5.1204379562043796</v>
       </c>
       <c r="W16" s="1">
@@ -9343,7 +9347,7 @@
         <v>4.9634146341463534</v>
       </c>
       <c r="Y16" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.1189707834213003</v>
       </c>
       <c r="Z16" s="1">
@@ -9360,7 +9364,7 @@
       </c>
       <c r="AC16" s="1"/>
       <c r="AD16" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.5812827273167684E-2</v>
       </c>
       <c r="AE16" s="1">
@@ -9403,19 +9407,19 @@
         <v>175.37500000000099</v>
       </c>
       <c r="AQ16" s="11">
-        <f t="shared" ref="AQ16:AS16" si="20">U2</f>
+        <f t="shared" ref="AQ16:AS16" si="22">U2</f>
         <v>26.543478260869758</v>
       </c>
       <c r="AR16" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>20.3333333333334</v>
       </c>
       <c r="AS16" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>18.223880597014915</v>
       </c>
     </row>
-    <row r="17" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="17" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B17" s="1">
         <v>33.628172839999998</v>
       </c>
@@ -9463,15 +9467,15 @@
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1">
-        <f>100/N17</f>
+        <f t="shared" si="17"/>
         <v>2.9851063829787274</v>
       </c>
       <c r="U17" s="1">
-        <f>100/O17</f>
+        <f t="shared" si="18"/>
         <v>2.93509615384616</v>
       </c>
       <c r="V17" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>4.0432276657060537</v>
       </c>
       <c r="W17" s="1">
@@ -9479,7 +9483,7 @@
         <v>2.1534391534391553</v>
       </c>
       <c r="Y17" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.12852921918749871</v>
       </c>
       <c r="Z17" s="1">
@@ -9496,7 +9500,7 @@
       </c>
       <c r="AC17" s="1"/>
       <c r="AD17" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.140928454309309E-2</v>
       </c>
       <c r="AE17" s="1">
@@ -9515,19 +9519,19 @@
         <v>38</v>
       </c>
       <c r="AJ17" s="12">
-        <f>AJ11/AJ$16</f>
+        <f t="shared" ref="AJ17:AM19" si="23">AJ11/AJ$16</f>
         <v>6.2193249727176723E-4</v>
       </c>
       <c r="AK17" s="12">
-        <f>AK11/AK$16</f>
+        <f t="shared" si="23"/>
         <v>5.2924374661365706E-4</v>
       </c>
       <c r="AL17" s="12">
-        <f>AL11/AL$16</f>
+        <f t="shared" si="23"/>
         <v>3.8785267279575455E-4</v>
       </c>
       <c r="AM17" s="12">
-        <f>AM11/AM$16</f>
+        <f t="shared" si="23"/>
         <v>3.0813553530232344E-3</v>
       </c>
       <c r="AN17" s="2"/>
@@ -9535,23 +9539,23 @@
         <v>38</v>
       </c>
       <c r="AP17" s="12">
-        <f>AP11/AP$16</f>
+        <f t="shared" ref="AP17:AS19" si="24">AP11/AP$16</f>
         <v>-4.4758420186870491E-3</v>
       </c>
       <c r="AQ17" s="12">
-        <f>AQ11/AQ$16</f>
+        <f t="shared" si="24"/>
         <v>-1.2085575272067276E-3</v>
       </c>
       <c r="AR17" s="12">
-        <f>AR11/AR$16</f>
+        <f t="shared" si="24"/>
         <v>-8.9661551101206688E-4</v>
       </c>
       <c r="AS17" s="12">
-        <f>AS11/AS$16</f>
+        <f t="shared" si="24"/>
         <v>-5.0776766938402263E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="18" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B18" s="1">
         <v>34.344647449999997</v>
       </c>
@@ -9599,15 +9603,15 @@
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
       <c r="T18" s="1">
-        <f>100/N18</f>
+        <f t="shared" si="17"/>
         <v>2.9107883817427416</v>
       </c>
       <c r="U18" s="1">
-        <f>100/O18</f>
+        <f t="shared" si="18"/>
         <v>1.1263837638376395</v>
       </c>
       <c r="V18" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>4.0316091954023152</v>
       </c>
       <c r="W18" s="1">
@@ -9615,7 +9619,7 @@
         <v>2.0350000000000015</v>
       </c>
       <c r="Y18" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>-1.0306220705601277E-2</v>
       </c>
       <c r="Z18" s="1">
@@ -9632,7 +9636,7 @@
       </c>
       <c r="AC18" s="1"/>
       <c r="AD18" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>8.7347606444954096E-4</v>
       </c>
       <c r="AE18" s="1">
@@ -9651,19 +9655,19 @@
         <v>36</v>
       </c>
       <c r="AJ18" s="12">
-        <f>AJ12/AJ$16</f>
+        <f t="shared" si="23"/>
         <v>1.452731495843273E-3</v>
       </c>
       <c r="AK18" s="12">
-        <f>AK12/AK$16</f>
+        <f t="shared" si="23"/>
         <v>1.6130940765402622E-3</v>
       </c>
       <c r="AL18" s="12">
-        <f>AL12/AL$16</f>
+        <f t="shared" si="23"/>
         <v>1.583531408465864E-3</v>
       </c>
       <c r="AM18" s="12">
-        <f>AM12/AM$16</f>
+        <f t="shared" si="23"/>
         <v>4.1735706014145828E-3</v>
       </c>
       <c r="AN18" s="1"/>
@@ -9671,23 +9675,23 @@
         <v>36</v>
       </c>
       <c r="AP18" s="12">
-        <f>AP12/AP$16</f>
+        <f t="shared" si="24"/>
         <v>7.9258996074493923E-2</v>
       </c>
       <c r="AQ18" s="12">
-        <f>AQ12/AQ$16</f>
+        <f t="shared" si="24"/>
         <v>2.5246429261307032E-2</v>
       </c>
       <c r="AR18" s="12">
-        <f>AR12/AR$16</f>
+        <f t="shared" si="24"/>
         <v>1.9729923185582272E-2</v>
       </c>
       <c r="AS18" s="12">
-        <f>AS12/AS$16</f>
+        <f t="shared" si="24"/>
         <v>4.7807376421932148E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="19" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B19" s="1">
         <v>34.655171420000002</v>
       </c>
@@ -9735,15 +9739,15 @@
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
       <c r="T19" s="1">
-        <f>100/N19</f>
+        <f t="shared" si="17"/>
         <v>2.8868312757201724</v>
       </c>
       <c r="U19" s="1">
-        <f>100/O19</f>
+        <f t="shared" si="18"/>
         <v>1.476420798065297</v>
       </c>
       <c r="V19" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>3.7214854111405873</v>
       </c>
       <c r="W19" s="1">
@@ -9751,7 +9755,7 @@
         <v>2.1197916666666701</v>
       </c>
       <c r="Y19" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>1.5114399330101946E-2</v>
       </c>
       <c r="Z19" s="1">
@@ -9768,7 +9772,7 @@
       </c>
       <c r="AC19" s="1"/>
       <c r="AD19" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.2590536682406395E-3</v>
       </c>
       <c r="AE19" s="1">
@@ -9787,19 +9791,19 @@
         <v>35</v>
       </c>
       <c r="AJ19" s="12">
-        <f>AJ13/AJ$16</f>
+        <f t="shared" si="23"/>
         <v>5.0189537839337992E-4</v>
       </c>
       <c r="AK19" s="12">
-        <f>AK13/AK$16</f>
+        <f t="shared" si="23"/>
         <v>5.3518083635148829E-4</v>
       </c>
       <c r="AL19" s="12">
-        <f>AL13/AL$16</f>
+        <f t="shared" si="23"/>
         <v>5.064618664839737E-4</v>
       </c>
       <c r="AM19" s="12">
-        <f>AM13/AM$16</f>
+        <f t="shared" si="23"/>
         <v>5.6706341312331033E-4</v>
       </c>
       <c r="AN19" s="2"/>
@@ -9807,23 +9811,23 @@
         <v>35</v>
       </c>
       <c r="AP19" s="12">
-        <f>AP13/AP$16</f>
+        <f t="shared" si="24"/>
         <v>1.6890489956909269E-2</v>
       </c>
       <c r="AQ19" s="12">
-        <f>AQ13/AQ$16</f>
+        <f t="shared" si="24"/>
         <v>4.6510429738779013E-3</v>
       </c>
       <c r="AR19" s="12">
-        <f>AR13/AR$16</f>
+        <f t="shared" si="24"/>
         <v>3.5855225878981827E-3</v>
       </c>
       <c r="AS19" s="12">
-        <f>AS13/AS$16</f>
+        <f t="shared" si="24"/>
         <v>1.1655654072936271E-2</v>
       </c>
     </row>
-    <row r="20" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="20" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B20" s="1">
         <v>35.427304530000001</v>
       </c>
@@ -9871,15 +9875,15 @@
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
       <c r="T20" s="1">
-        <f>100/N20</f>
+        <f t="shared" si="17"/>
         <v>2.8229376257545264</v>
       </c>
       <c r="U20" s="1">
-        <f>100/O20</f>
+        <f t="shared" si="18"/>
         <v>10.617391304347835</v>
       </c>
       <c r="V20" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>3.4303178484107604</v>
       </c>
       <c r="W20" s="1">
@@ -9887,7 +9891,7 @@
         <v>16.27999999999998</v>
       </c>
       <c r="Y20" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>3.2132969280027623E-3</v>
       </c>
       <c r="Z20" s="1">
@@ -9904,7 +9908,7 @@
       </c>
       <c r="AC20" s="1"/>
       <c r="AD20" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-2.5604366239884158E-4</v>
       </c>
       <c r="AE20" s="1">
@@ -9920,7 +9924,7 @@
         <v>-0.80198263867937847</v>
       </c>
     </row>
-    <row r="21" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="21" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B21" s="1">
         <v>39.17994487</v>
       </c>
@@ -9968,15 +9972,15 @@
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1">
-        <f>100/N21</f>
+        <f t="shared" si="17"/>
         <v>2.5555555555555616</v>
       </c>
       <c r="U21" s="1">
-        <f>100/O21</f>
+        <f t="shared" si="18"/>
         <v>6.529411764705932</v>
       </c>
       <c r="V21" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>3.1177777777777806</v>
       </c>
       <c r="W21" s="1">
@@ -9984,7 +9988,7 @@
         <v>11.201834862385343</v>
       </c>
       <c r="Y21" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>4.9510087391396951E-2</v>
       </c>
       <c r="Z21" s="1">
@@ -10001,7 +10005,7 @@
       </c>
       <c r="AC21" s="1"/>
       <c r="AD21" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.2293506105980363E-3</v>
       </c>
       <c r="AE21" s="1">
@@ -10056,7 +10060,7 @@
         <v>3.8564390310101624</v>
       </c>
     </row>
-    <row r="22" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="22" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B22" s="1">
         <v>45.118863169999997</v>
       </c>
@@ -10104,15 +10108,15 @@
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1">
-        <f>100/N22</f>
+        <f t="shared" si="17"/>
         <v>2.21993670886076</v>
       </c>
       <c r="U22" s="1">
-        <f>100/O22</f>
+        <f t="shared" si="18"/>
         <v>1.4872107186358108</v>
       </c>
       <c r="V22" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>2.7892644135188891</v>
       </c>
       <c r="W22" s="1">
@@ -10120,7 +10124,7 @@
         <v>2.0082236842105301</v>
       </c>
       <c r="Y22" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>7.2533875630796274E-2</v>
       </c>
       <c r="Z22" s="1">
@@ -10137,7 +10141,7 @@
       </c>
       <c r="AC22" s="1"/>
       <c r="AD22" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.5688091816954426E-3</v>
       </c>
       <c r="AE22" s="1">
@@ -10156,19 +10160,19 @@
         <v>38</v>
       </c>
       <c r="AJ22" s="12">
-        <f>AJ11/AJ$21</f>
+        <f t="shared" ref="AJ22:AM24" si="25">AJ11/AJ$21</f>
         <v>1.2077339803639494E-3</v>
       </c>
       <c r="AK22" s="12">
-        <f>AK11/AK$21</f>
+        <f t="shared" si="25"/>
         <v>1.0638140445615467E-3</v>
       </c>
       <c r="AL22" s="12">
-        <f>AL11/AL$21</f>
+        <f t="shared" si="25"/>
         <v>7.7326462511052895E-4</v>
       </c>
       <c r="AM22" s="12">
-        <f>AM11/AM$21</f>
+        <f t="shared" si="25"/>
         <v>5.9712851477868615E-3</v>
       </c>
       <c r="AN22" s="2"/>
@@ -10176,23 +10180,23 @@
         <v>38</v>
       </c>
       <c r="AP22" s="12">
-        <f>AP11/AP$21</f>
+        <f t="shared" ref="AP22:AS24" si="26">AP11/AP$21</f>
         <v>-6.2574333169052379E-2</v>
       </c>
       <c r="AQ22" s="12">
-        <f>AQ11/AQ$21</f>
+        <f t="shared" si="26"/>
         <v>-6.8932704027120911E-3</v>
       </c>
       <c r="AR22" s="12">
-        <f>AR11/AR$21</f>
+        <f t="shared" si="26"/>
         <v>-5.0561526865345718E-3</v>
       </c>
       <c r="AS22" s="12">
-        <f>AS11/AS$21</f>
+        <f t="shared" si="26"/>
         <v>-2.3994927194415146E-2</v>
       </c>
     </row>
-    <row r="23" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="23" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B23" s="1">
         <v>45.90439207</v>
       </c>
@@ -10240,15 +10244,15 @@
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1">
-        <f>100/N23</f>
+        <f t="shared" si="17"/>
         <v>2.1819595645412182</v>
       </c>
       <c r="U23" s="1">
-        <f>100/O23</f>
+        <f t="shared" si="18"/>
         <v>1.0872662511130908</v>
       </c>
       <c r="V23" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>2.5695970695970711</v>
       </c>
       <c r="W23" s="1">
@@ -10256,7 +10260,7 @@
         <v>1.1661891117478518</v>
       </c>
       <c r="Y23" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>7.4028563228900168E-2</v>
       </c>
       <c r="Z23" s="1">
@@ -10273,7 +10277,7 @@
       </c>
       <c r="AC23" s="1"/>
       <c r="AD23" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.5187772738658474E-3</v>
       </c>
       <c r="AE23" s="1">
@@ -10292,19 +10296,19 @@
         <v>36</v>
       </c>
       <c r="AJ23" s="12">
-        <f>AJ12/AJ$21</f>
+        <f t="shared" si="25"/>
         <v>2.8210669157366719E-3</v>
       </c>
       <c r="AK23" s="12">
-        <f>AK12/AK$21</f>
+        <f t="shared" si="25"/>
         <v>3.2424230702819373E-3</v>
       </c>
       <c r="AL23" s="12">
-        <f>AL12/AL$21</f>
+        <f t="shared" si="25"/>
         <v>3.1570978023475606E-3</v>
       </c>
       <c r="AM23" s="12">
-        <f>AM12/AM$21</f>
+        <f t="shared" si="25"/>
         <v>8.0878630635753436E-3</v>
       </c>
       <c r="AN23" s="1"/>
@@ -10312,23 +10316,23 @@
         <v>36</v>
       </c>
       <c r="AP23" s="12">
-        <f>AP12/AP$21</f>
+        <f t="shared" si="26"/>
         <v>1.1080772749134806</v>
       </c>
       <c r="AQ23" s="12">
-        <f>AQ12/AQ$21</f>
+        <f t="shared" si="26"/>
         <v>0.14399849381051746</v>
       </c>
       <c r="AR23" s="12">
-        <f>AR12/AR$21</f>
+        <f t="shared" si="26"/>
         <v>0.11126006955567823</v>
       </c>
       <c r="AS23" s="12">
-        <f>AS12/AS$21</f>
+        <f t="shared" si="26"/>
         <v>0.22591720303733792</v>
       </c>
     </row>
-    <row r="24" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="24" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B24" s="1">
         <v>50.232937120000003</v>
       </c>
@@ -10376,15 +10380,15 @@
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1">
-        <f>100/N24</f>
+        <f t="shared" si="17"/>
         <v>1.9957325746799446</v>
       </c>
       <c r="U24" s="1">
-        <f>100/O24</f>
+        <f t="shared" si="18"/>
         <v>12.210000000000015</v>
       </c>
       <c r="V24" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>2.5509090909090961</v>
       </c>
       <c r="W24" s="1">
@@ -10392,7 +10396,7 @@
         <v>1.1540642722117209</v>
       </c>
       <c r="Y24" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.12602336376340162</v>
       </c>
       <c r="Z24" s="1">
@@ -10409,7 +10413,7 @@
       </c>
       <c r="AC24" s="1"/>
       <c r="AD24" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.0068530062763461E-3</v>
       </c>
       <c r="AE24" s="1">
@@ -10428,19 +10432,19 @@
         <v>35</v>
       </c>
       <c r="AJ24" s="12">
-        <f>AJ13/AJ$21</f>
+        <f t="shared" si="25"/>
         <v>9.7463326925724869E-4</v>
       </c>
       <c r="AK24" s="12">
-        <f>AK13/AK$21</f>
+        <f t="shared" si="25"/>
         <v>1.075747977626112E-3</v>
       </c>
       <c r="AL24" s="12">
-        <f>AL13/AL$21</f>
+        <f t="shared" si="25"/>
         <v>1.009736615959181E-3</v>
       </c>
       <c r="AM24" s="12">
-        <f>AM13/AM$21</f>
+        <f t="shared" si="25"/>
         <v>1.0988986821381442E-3</v>
       </c>
       <c r="AN24" s="2"/>
@@ -10448,23 +10452,23 @@
         <v>35</v>
       </c>
       <c r="AP24" s="12">
-        <f>AP13/AP$21</f>
+        <f t="shared" si="26"/>
         <v>0.23613683001756383</v>
       </c>
       <c r="AQ24" s="12">
-        <f>AQ13/AQ$21</f>
+        <f t="shared" si="26"/>
         <v>2.6528233991206979E-2</v>
       </c>
       <c r="AR24" s="12">
-        <f>AR13/AR$21</f>
+        <f t="shared" si="26"/>
         <v>2.021931300850293E-2</v>
       </c>
       <c r="AS24" s="12">
-        <f>AS13/AS$21</f>
+        <f t="shared" si="26"/>
         <v>5.5079633412397501E-2</v>
       </c>
     </row>
-    <row r="25" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="25" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B25" s="1">
         <v>52.973726739999996</v>
       </c>
@@ -10512,15 +10516,15 @@
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1">
-        <f>100/N25</f>
+        <f t="shared" si="17"/>
         <v>1.8908355795148273</v>
       </c>
       <c r="U25" s="1">
-        <f>100/O25</f>
+        <f t="shared" si="18"/>
         <v>1.9918433931484505</v>
       </c>
       <c r="V25" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>2.2520064205457464</v>
       </c>
       <c r="W25" s="1">
@@ -10528,7 +10532,7 @@
         <v>1.0453767123287678</v>
       </c>
       <c r="Y25" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>8.7055321610897352E-2</v>
       </c>
       <c r="Z25" s="1">
@@ -10545,7 +10549,7 @@
       </c>
       <c r="AC25" s="1"/>
       <c r="AD25" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-3.1073384792408287E-3</v>
       </c>
       <c r="AE25" s="1">
@@ -10561,7 +10565,7 @@
         <v>-3.6422849611330577E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="26" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B26" s="1">
         <v>58.012670819999997</v>
       </c>
@@ -10609,15 +10613,15 @@
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1">
-        <f t="shared" ref="T26:T39" si="21">100/N26</f>
+        <f t="shared" ref="T26:T39" si="27">100/N26</f>
         <v>1.723587223587226</v>
       </c>
       <c r="U26" s="1">
-        <f t="shared" ref="U26:U39" si="22">100/O26</f>
+        <f t="shared" ref="U26:U39" si="28">100/O26</f>
         <v>12.852631578947387</v>
       </c>
       <c r="V26" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.948611111111114</v>
       </c>
       <c r="W26" s="1">
@@ -10625,7 +10629,7 @@
         <v>1.1110100090991812</v>
       </c>
       <c r="Y26" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>-5.860897747602678E-3</v>
       </c>
       <c r="Z26" s="1">
@@ -10642,7 +10646,7 @@
       </c>
       <c r="AC26" s="1"/>
       <c r="AD26" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>1.7413038106561807E-4</v>
       </c>
       <c r="AE26" s="1">
@@ -10658,7 +10662,7 @@
         <v>-3.9005634083317808E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="27" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B27" s="1">
         <v>62.685176329999997</v>
       </c>
@@ -10706,15 +10710,15 @@
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
       <c r="T27" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.5961319681456216</v>
       </c>
       <c r="U27" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>2.4817073170731767</v>
       </c>
       <c r="V27" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.6662707838479816</v>
       </c>
       <c r="W27" s="1">
@@ -10722,7 +10726,7 @@
         <v>18.223880597014915</v>
       </c>
       <c r="Y27" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>3.3715175331494152E-2</v>
       </c>
       <c r="Z27" s="1">
@@ -10739,7 +10743,7 @@
       </c>
       <c r="AC27" s="1"/>
       <c r="AD27" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-8.5847838849395508E-4</v>
       </c>
       <c r="AE27" s="1">
@@ -10755,7 +10759,7 @@
         <v>-0.87123591956983759</v>
       </c>
     </row>
-    <row r="28" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="28" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B28" s="1">
         <v>63.242376</v>
       </c>
@@ -10803,15 +10807,15 @@
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
       <c r="T28" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.5817361894024802</v>
       </c>
       <c r="U28" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>10.090909090909122</v>
       </c>
       <c r="V28" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.5997719498289644</v>
       </c>
       <c r="W28" s="1">
@@ -10819,7 +10823,7 @@
         <v>1.0654450261780113</v>
       </c>
       <c r="Y28" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>2.0708145402700495E-2</v>
       </c>
       <c r="Z28" s="1">
@@ -10836,7 +10840,7 @@
       </c>
       <c r="AC28" s="1"/>
       <c r="AD28" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.1792524365090742E-4</v>
       </c>
       <c r="AE28" s="1">
@@ -10860,7 +10864,7 @@
       <c r="AQ28" s="1"/>
       <c r="AR28" s="1"/>
     </row>
-    <row r="29" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="29" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B29" s="1">
         <v>68.567099420000005</v>
       </c>
@@ -10908,15 +10912,15 @@
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.4584199584199602</v>
       </c>
       <c r="U29" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>1.1573459715639811</v>
       </c>
       <c r="V29" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.5554323725055446</v>
       </c>
       <c r="W29" s="1">
@@ -10924,7 +10928,7 @@
         <v>2.7254464285714355</v>
       </c>
       <c r="Y29" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>-2.5624642898947059E-4</v>
       </c>
       <c r="Z29" s="1">
@@ -10941,7 +10945,7 @@
       </c>
       <c r="AC29" s="1"/>
       <c r="AD29" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>5.4503531501381985E-6</v>
       </c>
       <c r="AE29" s="1">
@@ -10965,7 +10969,7 @@
       <c r="AQ29" s="1"/>
       <c r="AR29" s="1"/>
     </row>
-    <row r="30" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="30" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B30" s="1">
         <v>70.527367060000003</v>
       </c>
@@ -11013,15 +11017,15 @@
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.4200404858299602</v>
       </c>
       <c r="U30" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>10.090909090909122</v>
       </c>
       <c r="V30" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.407221664994986</v>
       </c>
       <c r="W30" s="1">
@@ -11029,7 +11033,7 @@
         <v>2.4274353876739618</v>
       </c>
       <c r="Y30" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.10683961880260995</v>
       </c>
       <c r="Z30" s="1">
@@ -11046,7 +11050,7 @@
       </c>
       <c r="AC30" s="1"/>
       <c r="AD30" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-2.1511732326724431E-3</v>
       </c>
       <c r="AE30" s="1">
@@ -11070,7 +11074,7 @@
       <c r="AQ30" s="1"/>
       <c r="AR30" s="1"/>
     </row>
-    <row r="31" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="31" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B31" s="1">
         <v>73.09919721</v>
       </c>
@@ -11118,15 +11122,15 @@
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
       <c r="T31" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.3687804878048797</v>
       </c>
       <c r="U31" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>1.3242950108459872</v>
       </c>
       <c r="V31" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.312441534144061</v>
       </c>
       <c r="W31" s="1">
@@ -11134,7 +11138,7 @@
         <v>6.7833333333333528</v>
       </c>
       <c r="Y31" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>4.1463781632302243E-2</v>
       </c>
       <c r="Z31" s="1">
@@ -11151,7 +11155,7 @@
       </c>
       <c r="AC31" s="1"/>
       <c r="AD31" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-7.7640818798396793E-4</v>
       </c>
       <c r="AE31" s="1">
@@ -11175,7 +11179,7 @@
       <c r="AQ31" s="1"/>
       <c r="AR31" s="1"/>
     </row>
-    <row r="32" spans="2:45" x14ac:dyDescent="0.6">
+    <row r="32" spans="2:45" x14ac:dyDescent="0.45">
       <c r="B32" s="1">
         <v>74.649008069999994</v>
       </c>
@@ -11223,15 +11227,15 @@
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
       <c r="T32" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.3413001912045905</v>
       </c>
       <c r="U32" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>2.1960431654676276</v>
       </c>
       <c r="V32" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.2493321460374007</v>
       </c>
       <c r="W32" s="1">
@@ -11239,7 +11243,7 @@
         <v>1.2446483180428141</v>
       </c>
       <c r="Y32" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>9.4482054319399822E-2</v>
       </c>
       <c r="Z32" s="1">
@@ -11256,7 +11260,7 @@
       </c>
       <c r="AC32" s="1"/>
       <c r="AD32" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.6976621766384703E-3</v>
       </c>
       <c r="AE32" s="1">
@@ -11280,7 +11284,7 @@
       <c r="AQ32" s="1"/>
       <c r="AR32" s="1"/>
     </row>
-    <row r="33" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="33" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B33" s="1">
         <v>75.305004940000003</v>
       </c>
@@ -11328,15 +11332,15 @@
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
       <c r="T33" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.3298578199052151</v>
       </c>
       <c r="U33" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>5.3086956521739239</v>
       </c>
       <c r="V33" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.156636438582028</v>
       </c>
       <c r="W33" s="1">
@@ -11344,7 +11348,7 @@
         <v>2.184257602862258</v>
       </c>
       <c r="Y33" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.10899638689960511</v>
       </c>
       <c r="Z33" s="1">
@@ -11361,7 +11365,7 @@
       </c>
       <c r="AC33" s="1"/>
       <c r="AD33" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.9248348443154928E-3</v>
       </c>
       <c r="AE33" s="1">
@@ -11385,7 +11389,7 @@
       <c r="AQ33" s="1"/>
       <c r="AR33" s="1"/>
     </row>
-    <row r="34" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="34" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B34" s="1">
         <v>83.516144100000005</v>
       </c>
@@ -11433,15 +11437,15 @@
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
       <c r="T34" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.1970989761092163</v>
       </c>
       <c r="U34" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>6.7833333333333528</v>
       </c>
       <c r="V34" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.1490581490581495</v>
       </c>
       <c r="W34" s="1">
@@ -11449,7 +11453,7 @@
         <v>1.1900584795321643</v>
       </c>
       <c r="Y34" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>-1.9137439557994185E-2</v>
       </c>
       <c r="Z34" s="1">
@@ -11466,7 +11470,7 @@
       </c>
       <c r="AC34" s="1"/>
       <c r="AD34" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>2.7431114722920036E-4</v>
       </c>
       <c r="AE34" s="1">
@@ -11490,7 +11494,7 @@
       <c r="AQ34" s="1"/>
       <c r="AR34" s="1"/>
     </row>
-    <row r="35" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="35" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B35" s="1">
         <v>84.433256999999998</v>
       </c>
@@ -11538,15 +11542,15 @@
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
       <c r="T35" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.1859678782755718</v>
       </c>
       <c r="U35" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>1.5300751879699261</v>
       </c>
       <c r="V35" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.1305398871877521</v>
       </c>
       <c r="W35" s="1">
@@ -11554,7 +11558,7 @@
         <v>1.5416666666666683</v>
       </c>
       <c r="Y35" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.11394124803999262</v>
       </c>
       <c r="Z35" s="1">
@@ -11571,7 +11575,7 @@
       </c>
       <c r="AC35" s="1"/>
       <c r="AD35" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.6004435335956746E-3</v>
       </c>
       <c r="AE35" s="1">
@@ -11595,7 +11599,7 @@
       <c r="AQ35" s="1"/>
       <c r="AR35" s="1"/>
     </row>
-    <row r="36" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="36" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B36" s="1">
         <v>92.083094310000007</v>
       </c>
@@ -11643,15 +11647,15 @@
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
       <c r="T36" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.085913312693499</v>
       </c>
       <c r="U36" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>4.943319838056687</v>
       </c>
       <c r="V36" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.10996835443038</v>
       </c>
       <c r="W36" s="1">
@@ -11659,7 +11663,7 @@
         <v>2.3941176470588275</v>
       </c>
       <c r="Y36" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>-5.2877284888950271E-3</v>
       </c>
       <c r="Z36" s="1">
@@ -11676,7 +11680,7 @@
       </c>
       <c r="AC36" s="1"/>
       <c r="AD36" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>6.2356883237191241E-5</v>
       </c>
       <c r="AE36" s="1">
@@ -11700,7 +11704,7 @@
       <c r="AQ36" s="1"/>
       <c r="AR36" s="1"/>
     </row>
-    <row r="37" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="37" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B37" s="1">
         <v>94.165881420000005</v>
       </c>
@@ -11748,15 +11752,15 @@
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.0628787878787889</v>
       </c>
       <c r="U37" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>1.362723214285716</v>
       </c>
       <c r="V37" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.0825617283950619</v>
       </c>
       <c r="W37" s="1">
@@ -11764,7 +11768,7 @@
         <v>2.0418060200668928</v>
       </c>
       <c r="Y37" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>8.1775931760603271E-2</v>
       </c>
       <c r="Z37" s="1">
@@ -11781,7 +11785,7 @@
       </c>
       <c r="AC37" s="1"/>
       <c r="AD37" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-9.2302967823032489E-4</v>
       </c>
       <c r="AE37" s="1">
@@ -11805,7 +11809,7 @@
       <c r="AQ37" s="1"/>
       <c r="AR37" s="1"/>
     </row>
-    <row r="38" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="38" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B38" s="1">
         <v>97.159661510000007</v>
       </c>
@@ -11853,15 +11857,15 @@
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
       <c r="T38" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.0293470286133537</v>
       </c>
       <c r="U38" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>1.2934322033898307</v>
       </c>
       <c r="V38" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.0808936825885989</v>
       </c>
       <c r="W38" s="1">
@@ -11869,7 +11873,7 @@
         <v>1.2210000000000001</v>
       </c>
       <c r="Y38" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>1.0695009643711728E-2</v>
       </c>
       <c r="Z38" s="1">
@@ -11886,7 +11890,7 @@
       </c>
       <c r="AC38" s="1"/>
       <c r="AD38" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-1.133070682486359E-4</v>
       </c>
       <c r="AE38" s="1">
@@ -11910,7 +11914,7 @@
       <c r="AQ38" s="1"/>
       <c r="AR38" s="1"/>
     </row>
-    <row r="39" spans="2:44" x14ac:dyDescent="0.6">
+    <row r="39" spans="2:44" x14ac:dyDescent="0.45">
       <c r="B39" s="1">
         <v>99.480866559999996</v>
       </c>
@@ -11958,15 +11962,15 @@
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
       <c r="T39" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="27"/>
         <v>1.0057347670250905</v>
       </c>
       <c r="U39" s="1">
-        <f t="shared" si="22"/>
+        <f t="shared" si="28"/>
         <v>3.075566750629724</v>
       </c>
       <c r="V39" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>1.0064562410329996</v>
       </c>
       <c r="W39" s="1">
@@ -11974,7 +11978,7 @@
         <v>4.5559701492537412</v>
       </c>
       <c r="Y39" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>5.1073259928799075E-2</v>
       </c>
       <c r="Z39" s="1">
@@ -11991,7 +11995,7 @@
       </c>
       <c r="AC39" s="1"/>
       <c r="AD39" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>-5.1634203593042827E-4</v>
       </c>
       <c r="AE39" s="1">

</xml_diff>